<commit_message>
docs: update Test Plan tracking for Milestone 2
</commit_message>
<xml_diff>
--- a/docs/agile/Defect_Tracker Template_v0.1.xlsx
+++ b/docs/agile/Defect_Tracker Template_v0.1.xlsx
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:K22"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="17.5703125" defaultRowHeight="12.75"/>
   <cols>
     <col width="6.140625" bestFit="1" customWidth="1" style="4" min="1" max="1"/>
@@ -1020,6 +1020,116 @@
       <c r="I20" s="3" t="n"/>
       <c r="J20" s="3" t="n"/>
       <c r="K20" s="6" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>5</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Gyana</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Gemini free-tier RPM limit (15 requests/min) hit during M2.4 validation suite run, in addition to a separate daily quota exhaustion on gemini-3.7-flash (20/day).</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Gyana</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Configuration/Logical</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Switched LLM_MODEL to gemini-2.0-flash-lite (1500/day free tier). Optimized run_validation_suite.py to skip unnecessary Accuracy calls for irrelevant/off-topic cases (24-&gt;22 calls) and added configurable delay between calls. Updated LLMClient to parse Gemini's actual retry_delay from 429 errors instead of blind exponential backoff.</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Confirmed fixed - validation suite completed successfully with 0/22 mismatches.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>6</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Gyana</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>M2.4 validation run found 3 prompt-quality mismatches: (1) Accuracy agent classified a multi-claim response as 'incorrect' when it should be 'partially_correct' since one claim was right; (2) Relevance agent had no clear distinction between 'unrelated' and 'off_topic' categories; (3) Hallucination agent flagged an off-topic response as having unsupported claims when it wasn't attempting to answer the question at all.</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Gyana</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Logical (prompt design)</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Rewrote Accuracy prompt with explicit multi-claim partial-correctness rule and example. Rewrote Relevance prompt with explicit unrelated-vs-off_topic definitions and examples. Rewrote Hallucination prompt to first check whether the response attempts to answer the question before evaluating claims for support.</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Re-ran validation suite after fix: 0/22 mismatches, confirmed resolved.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
complete Milestone 3 evaluation system
</commit_message>
<xml_diff>
--- a/docs/agile/Defect_Tracker Template_v0.1.xlsx
+++ b/docs/agile/Defect_Tracker Template_v0.1.xlsx
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K22"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="17.5703125" defaultRowHeight="12.75"/>
   <cols>
     <col width="6.140625" bestFit="1" customWidth="1" style="4" min="1" max="1"/>
@@ -1128,6 +1128,61 @@
       <c r="K22" t="inlineStr">
         <is>
           <t>Re-ran validation suite after fix: 0/22 mismatches, confirmed resolved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>7</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Gyana</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>FastAPI's UploadFile/File-based CSV upload endpoint (POST /evaluate/batch) requires the python-multipart package to parse multipart form data. This was not present in requirements.txt, since no prior milestone needed file uploads.</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Gyana</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Configuration/Dependency</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Added python-multipart==0.0.12 to requirements.txt.</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Confirmed fixed — batch CSV upload endpoint works correctly after installing the dependency; low severity, caught during initial implementation before manual testing.</t>
         </is>
       </c>
     </row>

</xml_diff>